<commit_message>
Add PiN results step2 hybrid for Central_African_Republic___CAR
</commit_message>
<xml_diff>
--- a/platform_PiN_output/Central_African_Republic___CAR/PiN_step2_Central_African_Republic___CAR_1010_09AM.xlsx
+++ b/platform_PiN_output/Central_African_Republic___CAR/PiN_step2_Central_African_Republic___CAR_1010_09AM.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PiN TOTAL" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall PiN and severity" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PiN total par admin" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PiN -- hote" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PiN -- idp_host" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PiN -- retourne" sheetId="5" state="visible" r:id="rId5"/>
@@ -191,56 +191,34 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -609,22 +587,22 @@
   <dimension ref="A1:T14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="33" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="23" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="33" customWidth="1" min="19" max="19"/>
-    <col width="33" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="27" customWidth="1" min="11" max="11"/>
+    <col width="27" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="24" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="37" customWidth="1" min="19" max="19"/>
+    <col width="37" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -666,12 +644,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Population group</t>
+          <t>Groupe de population</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="F5" s="7" t="n"/>
@@ -683,62 +661,62 @@
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>Population group</t>
+          <t>Groupe de population</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>TotN</t>
+          <t>Population totale</t>
         </is>
       </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>% severity levels 1-2</t>
+          <t>% niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t># severity levels 1-2</t>
+          <t># niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="M5" s="6" t="inlineStr">
         <is>
-          <t>% severity level 3</t>
+          <t>% niveau de sévérité 3</t>
         </is>
       </c>
       <c r="N5" s="6" t="inlineStr">
         <is>
-          <t># severity level 3</t>
+          <t># niveau de sévérité 3</t>
         </is>
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>% severity level 4</t>
+          <t>% niveau de sévérité 4</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
         <is>
-          <t># severity level 4</t>
+          <t># niveau de sévérité 4</t>
         </is>
       </c>
       <c r="Q5" s="6" t="inlineStr">
         <is>
-          <t>% severity level 5</t>
+          <t>% niveau de sévérité 5</t>
         </is>
       </c>
       <c r="R5" s="6" t="inlineStr">
         <is>
-          <t># severity level 5</t>
+          <t># niveau de sévérité 5</t>
         </is>
       </c>
       <c r="S5" s="6" t="inlineStr">
         <is>
-          <t>% Tot PiN (severity levels 3-5)</t>
+          <t>% Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="T5" s="6" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
     </row>
@@ -747,12 +725,12 @@
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>TOTAL (5-17 y.o.)</t>
+          <t>TOTAL (5-17 ans)</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>All population groups</t>
+          <t>Tous les groupes de population</t>
         </is>
       </c>
       <c r="E6" s="9" t="n">
@@ -762,12 +740,12 @@
       <c r="G6" s="10" t="n"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>TOTAL (5-17 y.o.)</t>
+          <t>TOTAL (5-17 ans)</t>
         </is>
       </c>
       <c r="I6" s="9" t="inlineStr">
         <is>
-          <t>All population groups</t>
+          <t>Tous les groupes de population</t>
         </is>
       </c>
       <c r="J6" s="9" t="n">
@@ -809,7 +787,7 @@
       <c r="B7" s="2" t="n"/>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>hote (5-17 y.o.)</t>
+          <t>hote (5-17 ans)</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
@@ -824,7 +802,7 @@
       <c r="G7" s="4" t="n"/>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>hote (5-17 y.o.)</t>
+          <t>hote (5-17 ans)</t>
         </is>
       </c>
       <c r="I7" s="11" t="inlineStr">
@@ -871,7 +849,7 @@
       <c r="B8" s="2" t="n"/>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>idp_host (5-17 y.o.)</t>
+          <t>idp_host (5-17 ans)</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
@@ -886,7 +864,7 @@
       <c r="G8" s="4" t="n"/>
       <c r="H8" s="11" t="inlineStr">
         <is>
-          <t>idp_host (5-17 y.o.)</t>
+          <t>idp_host (5-17 ans)</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -933,7 +911,7 @@
       <c r="B9" s="2" t="n"/>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>retourne (5-17 y.o.)</t>
+          <t>retourne (5-17 ans)</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
@@ -948,7 +926,7 @@
       <c r="G9" s="4" t="n"/>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>retourne (5-17 y.o.)</t>
+          <t>retourne (5-17 ans)</t>
         </is>
       </c>
       <c r="I9" s="11" t="inlineStr">
@@ -995,7 +973,7 @@
       <c r="B10" s="2" t="n"/>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>idp_site (5-17 y.o.)</t>
+          <t>idp_site (5-17 ans)</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -1010,7 +988,7 @@
       <c r="G10" s="4" t="n"/>
       <c r="H10" s="11" t="inlineStr">
         <is>
-          <t>idp_site (5-17 y.o.)</t>
+          <t>idp_site (5-17 ans)</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -1057,12 +1035,12 @@
       <c r="B11" s="2" t="n"/>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>Girls (5-17 y.o.)</t>
+          <t>Filles (5-17 ans)</t>
         </is>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
-          <t>All population groups</t>
+          <t>Tous les groupes de population</t>
         </is>
       </c>
       <c r="E11" s="12" t="n">
@@ -1089,12 +1067,12 @@
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="12" t="inlineStr">
         <is>
-          <t>Boys (5-17 y.o.)</t>
+          <t>Garcons (5-17 ans)</t>
         </is>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>All population groups</t>
+          <t>Tous les groupes de population</t>
         </is>
       </c>
       <c r="E12" s="12" t="n">
@@ -1121,12 +1099,12 @@
       <c r="B13" s="2" t="n"/>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>ECE (5 y.o.)</t>
+          <t>Éducation préscolaire (5 ans)</t>
         </is>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>All population groups</t>
+          <t>Tous les groupes de population</t>
         </is>
       </c>
       <c r="E13" s="13" t="n">
@@ -1153,12 +1131,12 @@
       <c r="B14" s="2" t="n"/>
       <c r="C14" s="13" t="inlineStr">
         <is>
-          <t>Children with disability</t>
+          <t>Enfants en situation de handicap</t>
         </is>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>All population groups</t>
+          <t>Tous les groupes de population</t>
         </is>
       </c>
       <c r="E14" s="13" t="n">
@@ -1197,25 +1175,25 @@
   <dimension ref="A1:Q68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="33" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="37" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Overall PiN and severity (5-17 y.o.)</t>
+          <t>PiN total par admin (5-17 ans)</t>
         </is>
       </c>
     </row>
@@ -1234,62 +1212,62 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>TotN</t>
+          <t>Population totale</t>
         </is>
       </c>
       <c r="G5" s="16" t="inlineStr">
         <is>
-          <t>% severity levels 1-2</t>
+          <t>% niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t># severity levels 1-2</t>
+          <t># niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="I5" s="17" t="inlineStr">
         <is>
-          <t>% severity level 3</t>
+          <t>% niveau de sévérité 3</t>
         </is>
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t># severity level 3</t>
+          <t># niveau de sévérité 3</t>
         </is>
       </c>
       <c r="K5" s="18" t="inlineStr">
         <is>
-          <t>% severity level 4</t>
+          <t>% niveau de sévérité 4</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t># severity level 4</t>
+          <t># niveau de sévérité 4</t>
         </is>
       </c>
       <c r="M5" s="19" t="inlineStr">
         <is>
-          <t>% severity level 5</t>
+          <t>% niveau de sévérité 5</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t># severity level 5</t>
+          <t># niveau de sévérité 5</t>
         </is>
       </c>
       <c r="O5" s="20" t="inlineStr">
         <is>
-          <t>% Tot PiN (severity levels 3-5)</t>
+          <t>% Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="P5" s="20" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="Q5" s="20" t="inlineStr">
         <is>
-          <t>Area severity</t>
+          <t>Sévérité de la zone</t>
         </is>
       </c>
     </row>
@@ -4377,26 +4355,26 @@
   <dimension ref="A1:R66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="33" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="37" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>PiN -- hote (5-17 y.o.)</t>
+          <t>PiN -- hote (5-17 ans)</t>
         </is>
       </c>
     </row>
@@ -4415,67 +4393,67 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Population group</t>
+          <t>Groupe de population</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>TotN</t>
+          <t>Population totale</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>% severity levels 1-2</t>
+          <t>% niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t># severity levels 1-2</t>
+          <t># niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>% severity level 3</t>
+          <t>% niveau de sévérité 3</t>
         </is>
       </c>
       <c r="K5" s="17" t="inlineStr">
         <is>
-          <t># severity level 3</t>
+          <t># niveau de sévérité 3</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>% severity level 4</t>
+          <t>% niveau de sévérité 4</t>
         </is>
       </c>
       <c r="M5" s="18" t="inlineStr">
         <is>
-          <t># severity level 4</t>
+          <t># niveau de sévérité 4</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>% severity level 5</t>
+          <t>% niveau de sévérité 5</t>
         </is>
       </c>
       <c r="O5" s="19" t="inlineStr">
         <is>
-          <t># severity level 5</t>
+          <t># niveau de sévérité 5</t>
         </is>
       </c>
       <c r="P5" s="20" t="inlineStr">
         <is>
-          <t>% Tot PiN (severity levels 3-5)</t>
+          <t>% Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="Q5" s="20" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="R5" s="20" t="inlineStr">
         <is>
-          <t>Area severity</t>
+          <t>Sévérité de la zone</t>
         </is>
       </c>
     </row>
@@ -7790,26 +7768,26 @@
   <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="33" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="37" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>PiN -- idp_host (5-17 y.o.)</t>
+          <t>PiN -- idp_host (5-17 ans)</t>
         </is>
       </c>
     </row>
@@ -7828,67 +7806,67 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Population group</t>
+          <t>Groupe de population</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>TotN</t>
+          <t>Population totale</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>% severity levels 1-2</t>
+          <t>% niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t># severity levels 1-2</t>
+          <t># niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>% severity level 3</t>
+          <t>% niveau de sévérité 3</t>
         </is>
       </c>
       <c r="K5" s="17" t="inlineStr">
         <is>
-          <t># severity level 3</t>
+          <t># niveau de sévérité 3</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>% severity level 4</t>
+          <t>% niveau de sévérité 4</t>
         </is>
       </c>
       <c r="M5" s="18" t="inlineStr">
         <is>
-          <t># severity level 4</t>
+          <t># niveau de sévérité 4</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>% severity level 5</t>
+          <t>% niveau de sévérité 5</t>
         </is>
       </c>
       <c r="O5" s="19" t="inlineStr">
         <is>
-          <t># severity level 5</t>
+          <t># niveau de sévérité 5</t>
         </is>
       </c>
       <c r="P5" s="20" t="inlineStr">
         <is>
-          <t>% Tot PiN (severity levels 3-5)</t>
+          <t>% Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="Q5" s="20" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="R5" s="20" t="inlineStr">
         <is>
-          <t>Area severity</t>
+          <t>Sévérité de la zone</t>
         </is>
       </c>
     </row>
@@ -10879,26 +10857,26 @@
   <dimension ref="A1:R60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="33" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="37" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>PiN -- retourne (5-17 y.o.)</t>
+          <t>PiN -- retourne (5-17 ans)</t>
         </is>
       </c>
     </row>
@@ -10917,67 +10895,67 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Population group</t>
+          <t>Groupe de population</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>TotN</t>
+          <t>Population totale</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>% severity levels 1-2</t>
+          <t>% niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t># severity levels 1-2</t>
+          <t># niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>% severity level 3</t>
+          <t>% niveau de sévérité 3</t>
         </is>
       </c>
       <c r="K5" s="17" t="inlineStr">
         <is>
-          <t># severity level 3</t>
+          <t># niveau de sévérité 3</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>% severity level 4</t>
+          <t>% niveau de sévérité 4</t>
         </is>
       </c>
       <c r="M5" s="18" t="inlineStr">
         <is>
-          <t># severity level 4</t>
+          <t># niveau de sévérité 4</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>% severity level 5</t>
+          <t>% niveau de sévérité 5</t>
         </is>
       </c>
       <c r="O5" s="19" t="inlineStr">
         <is>
-          <t># severity level 5</t>
+          <t># niveau de sévérité 5</t>
         </is>
       </c>
       <c r="P5" s="20" t="inlineStr">
         <is>
-          <t>% Tot PiN (severity levels 3-5)</t>
+          <t>% Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="Q5" s="20" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="R5" s="20" t="inlineStr">
         <is>
-          <t>Area severity</t>
+          <t>Sévérité de la zone</t>
         </is>
       </c>
     </row>
@@ -13968,26 +13946,26 @@
   <dimension ref="A1:R25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="23" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="33" customWidth="1" min="16" max="16"/>
-    <col width="33" customWidth="1" min="17" max="17"/>
-    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="37" customWidth="1" min="16" max="16"/>
+    <col width="37" customWidth="1" min="17" max="17"/>
+    <col width="21" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>PiN -- idp_site (5-17 y.o.)</t>
+          <t>PiN -- idp_site (5-17 ans)</t>
         </is>
       </c>
     </row>
@@ -14006,67 +13984,67 @@
       </c>
       <c r="F5" s="15" t="inlineStr">
         <is>
-          <t>Population group</t>
+          <t>Groupe de population</t>
         </is>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>TotN</t>
+          <t>Population totale</t>
         </is>
       </c>
       <c r="H5" s="16" t="inlineStr">
         <is>
-          <t>% severity levels 1-2</t>
+          <t>% niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="I5" s="16" t="inlineStr">
         <is>
-          <t># severity levels 1-2</t>
+          <t># niveaux de sévérité 1-2</t>
         </is>
       </c>
       <c r="J5" s="17" t="inlineStr">
         <is>
-          <t>% severity level 3</t>
+          <t>% niveau de sévérité 3</t>
         </is>
       </c>
       <c r="K5" s="17" t="inlineStr">
         <is>
-          <t># severity level 3</t>
+          <t># niveau de sévérité 3</t>
         </is>
       </c>
       <c r="L5" s="18" t="inlineStr">
         <is>
-          <t>% severity level 4</t>
+          <t>% niveau de sévérité 4</t>
         </is>
       </c>
       <c r="M5" s="18" t="inlineStr">
         <is>
-          <t># severity level 4</t>
+          <t># niveau de sévérité 4</t>
         </is>
       </c>
       <c r="N5" s="19" t="inlineStr">
         <is>
-          <t>% severity level 5</t>
+          <t>% niveau de sévérité 5</t>
         </is>
       </c>
       <c r="O5" s="19" t="inlineStr">
         <is>
-          <t># severity level 5</t>
+          <t># niveau de sévérité 5</t>
         </is>
       </c>
       <c r="P5" s="20" t="inlineStr">
         <is>
-          <t>% Tot PiN (severity levels 3-5)</t>
+          <t>% Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="Q5" s="20" t="inlineStr">
         <is>
-          <t># Tot PiN (severity levels 3-5)</t>
+          <t># Tot PiN (niveaux de sévérité 3-5)</t>
         </is>
       </c>
       <c r="R5" s="20" t="inlineStr">
         <is>
-          <t>Area severity</t>
+          <t>Sévérité de la zone</t>
         </is>
       </c>
     </row>

</xml_diff>